<commit_message>
upload project to render
</commit_message>
<xml_diff>
--- a/audit_log.xlsx
+++ b/audit_log.xlsx
@@ -417,7 +417,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F2"/>
+  <dimension ref="A1:F17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -454,7 +454,7 @@
     </row>
     <row r="2">
       <c r="A2" s="1" t="n">
-        <v>46190.47405079143</v>
+        <v>46190.47405078704</v>
       </c>
       <c r="B2" t="inlineStr">
         <is>
@@ -471,6 +471,336 @@
         <v>0</v>
       </c>
       <c r="F2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="1" t="n">
+        <v>46191.4581020949</v>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>joanine</t>
+        </is>
+      </c>
+      <c r="C3" t="n">
+        <v>226</v>
+      </c>
+      <c r="D3" t="n">
+        <v>197</v>
+      </c>
+      <c r="E3" t="n">
+        <v>29</v>
+      </c>
+      <c r="F3" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="1" t="n">
+        <v>46191.46680469908</v>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>joanine</t>
+        </is>
+      </c>
+      <c r="C4" t="n">
+        <v>5</v>
+      </c>
+      <c r="D4" t="n">
+        <v>5</v>
+      </c>
+      <c r="E4" t="n">
+        <v>0</v>
+      </c>
+      <c r="F4" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="1" t="n">
+        <v>46191.47738082176</v>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>joanine</t>
+        </is>
+      </c>
+      <c r="C5" t="n">
+        <v>5</v>
+      </c>
+      <c r="D5" t="n">
+        <v>5</v>
+      </c>
+      <c r="E5" t="n">
+        <v>0</v>
+      </c>
+      <c r="F5" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="1" t="n">
+        <v>46191.48135388889</v>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>joanine</t>
+        </is>
+      </c>
+      <c r="C6" t="n">
+        <v>5</v>
+      </c>
+      <c r="D6" t="n">
+        <v>5</v>
+      </c>
+      <c r="E6" t="n">
+        <v>0</v>
+      </c>
+      <c r="F6" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="1" t="n">
+        <v>46191.53241659722</v>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>joanine</t>
+        </is>
+      </c>
+      <c r="C7" t="n">
+        <v>5</v>
+      </c>
+      <c r="D7" t="n">
+        <v>5</v>
+      </c>
+      <c r="E7" t="n">
+        <v>0</v>
+      </c>
+      <c r="F7" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="1" t="n">
+        <v>46191.53557599537</v>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>joanine</t>
+        </is>
+      </c>
+      <c r="C8" t="n">
+        <v>5</v>
+      </c>
+      <c r="D8" t="n">
+        <v>5</v>
+      </c>
+      <c r="E8" t="n">
+        <v>0</v>
+      </c>
+      <c r="F8" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="1" t="n">
+        <v>46191.54286517361</v>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>joanine</t>
+        </is>
+      </c>
+      <c r="C9" t="n">
+        <v>5</v>
+      </c>
+      <c r="D9" t="n">
+        <v>5</v>
+      </c>
+      <c r="E9" t="n">
+        <v>0</v>
+      </c>
+      <c r="F9" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="1" t="n">
+        <v>46191.54344265047</v>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>joanine</t>
+        </is>
+      </c>
+      <c r="C10" t="n">
+        <v>226</v>
+      </c>
+      <c r="D10" t="n">
+        <v>197</v>
+      </c>
+      <c r="E10" t="n">
+        <v>29</v>
+      </c>
+      <c r="F10" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="1" t="n">
+        <v>46191.54821824074</v>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>joanine</t>
+        </is>
+      </c>
+      <c r="C11" t="n">
+        <v>226</v>
+      </c>
+      <c r="D11" t="n">
+        <v>197</v>
+      </c>
+      <c r="E11" t="n">
+        <v>29</v>
+      </c>
+      <c r="F11" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="1" t="n">
+        <v>46191.55566244213</v>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>joanine</t>
+        </is>
+      </c>
+      <c r="C12" t="n">
+        <v>226</v>
+      </c>
+      <c r="D12" t="n">
+        <v>197</v>
+      </c>
+      <c r="E12" t="n">
+        <v>29</v>
+      </c>
+      <c r="F12" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="1" t="n">
+        <v>46191.5637594213</v>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>joanine</t>
+        </is>
+      </c>
+      <c r="C13" t="n">
+        <v>234</v>
+      </c>
+      <c r="D13" t="n">
+        <v>205</v>
+      </c>
+      <c r="E13" t="n">
+        <v>29</v>
+      </c>
+      <c r="F13" t="n">
+        <v>2.91038304567337e-11</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="1" t="n">
+        <v>46191.62378143518</v>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>joanine</t>
+        </is>
+      </c>
+      <c r="C14" t="n">
+        <v>5</v>
+      </c>
+      <c r="D14" t="n">
+        <v>5</v>
+      </c>
+      <c r="E14" t="n">
+        <v>0</v>
+      </c>
+      <c r="F14" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="1" t="n">
+        <v>46191.62881827547</v>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>joanine</t>
+        </is>
+      </c>
+      <c r="C15" t="n">
+        <v>5</v>
+      </c>
+      <c r="D15" t="n">
+        <v>5</v>
+      </c>
+      <c r="E15" t="n">
+        <v>0</v>
+      </c>
+      <c r="F15" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="1" t="n">
+        <v>46191.62905206018</v>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>joanine</t>
+        </is>
+      </c>
+      <c r="C16" t="n">
+        <v>5</v>
+      </c>
+      <c r="D16" t="n">
+        <v>5</v>
+      </c>
+      <c r="E16" t="n">
+        <v>0</v>
+      </c>
+      <c r="F16" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="1" t="n">
+        <v>46191.63320799375</v>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>joanine</t>
+        </is>
+      </c>
+      <c r="C17" t="n">
+        <v>5</v>
+      </c>
+      <c r="D17" t="n">
+        <v>5</v>
+      </c>
+      <c r="E17" t="n">
+        <v>0</v>
+      </c>
+      <c r="F17" t="n">
         <v>0</v>
       </c>
     </row>

</xml_diff>